<commit_message>
Improve output caching and implement T2 and T3 signatures.
</commit_message>
<xml_diff>
--- a/PrefixesV2.xlsx
+++ b/PrefixesV2.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matty\source\repos\SortNetSAT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{506CC8DD-91E3-4722-9805-B8DA5A54A99D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DFB5BC2-A680-4F98-BFE8-FBADAB65BB90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{0104B856-7785-45C9-88AA-D6349C4CC1CA}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{0104B856-7785-45C9-88AA-D6349C4CC1CA}"/>
   </bookViews>
   <sheets>
     <sheet name="1sym" sheetId="7" r:id="rId1"/>
     <sheet name="2sym" sheetId="1" r:id="rId2"/>
     <sheet name="3sym" sheetId="8" r:id="rId3"/>
+    <sheet name="Combined" sheetId="9" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,12 +42,21 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="5">
   <si>
     <t>Subsumption</t>
   </si>
   <si>
     <t>n</t>
+  </si>
+  <si>
+    <t>depth 1</t>
+  </si>
+  <si>
+    <t>depth 2</t>
+  </si>
+  <si>
+    <t>depth 3</t>
   </si>
 </sst>
 </file>
@@ -76,7 +86,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -93,16 +103,43 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -663,4 +700,139 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6AEAF64-B24F-4E2D-89CC-9E6FA66706DC}">
+  <dimension ref="A1:K4"/>
+  <sheetFormatPr defaultRowHeight="12" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="18.83203125" style="6" customWidth="1"/>
+    <col min="2" max="16384" width="9.33203125" style="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="3">
+        <v>2</v>
+      </c>
+      <c r="C1" s="3">
+        <v>4</v>
+      </c>
+      <c r="D1" s="3">
+        <v>6</v>
+      </c>
+      <c r="E1" s="3">
+        <v>8</v>
+      </c>
+      <c r="F1" s="3">
+        <v>10</v>
+      </c>
+      <c r="G1" s="3">
+        <v>12</v>
+      </c>
+      <c r="H1" s="3">
+        <v>14</v>
+      </c>
+      <c r="I1" s="3">
+        <v>16</v>
+      </c>
+      <c r="J1" s="3">
+        <v>18</v>
+      </c>
+      <c r="K1" s="5"/>
+    </row>
+    <row r="2" spans="1:11" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="4">
+        <v>1</v>
+      </c>
+      <c r="C2" s="4">
+        <v>2</v>
+      </c>
+      <c r="D2" s="4">
+        <v>2</v>
+      </c>
+      <c r="E2" s="4">
+        <v>3</v>
+      </c>
+      <c r="F2" s="4">
+        <v>3</v>
+      </c>
+      <c r="G2" s="4">
+        <v>4</v>
+      </c>
+      <c r="H2" s="4">
+        <v>4</v>
+      </c>
+      <c r="I2" s="4">
+        <v>5</v>
+      </c>
+      <c r="J2" s="4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A3" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="4">
+        <v>1</v>
+      </c>
+      <c r="C3" s="4">
+        <v>2</v>
+      </c>
+      <c r="D3" s="4">
+        <v>4</v>
+      </c>
+      <c r="E3" s="4">
+        <v>12</v>
+      </c>
+      <c r="F3" s="4">
+        <v>18</v>
+      </c>
+      <c r="G3" s="4">
+        <v>41</v>
+      </c>
+      <c r="H3" s="4">
+        <v>69</v>
+      </c>
+      <c r="I3" s="4">
+        <v>149</v>
+      </c>
+      <c r="J3" s="4"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A4" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="4">
+        <v>1</v>
+      </c>
+      <c r="C4" s="4">
+        <v>1</v>
+      </c>
+      <c r="D4" s="4">
+        <v>3</v>
+      </c>
+      <c r="E4" s="4">
+        <v>13</v>
+      </c>
+      <c r="F4" s="4">
+        <v>171</v>
+      </c>
+      <c r="G4" s="4">
+        <v>1502</v>
+      </c>
+      <c r="H4" s="4"/>
+      <c r="I4" s="4"/>
+      <c r="J4" s="4"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Applying the same caching strategy to signatures.
</commit_message>
<xml_diff>
--- a/PrefixesV2.xlsx
+++ b/PrefixesV2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matty\source\repos\SortNetSAT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DFB5BC2-A680-4F98-BFE8-FBADAB65BB90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6E74410-24F9-4943-89B7-A1A6D678896B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{0104B856-7785-45C9-88AA-D6349C4CC1CA}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="10">
   <si>
     <t>Subsumption</t>
   </si>
@@ -58,12 +58,27 @@
   <si>
     <t>depth 3</t>
   </si>
+  <si>
+    <t>depth 4</t>
+  </si>
+  <si>
+    <t>depth 5</t>
+  </si>
+  <si>
+    <t>depth 6</t>
+  </si>
+  <si>
+    <t>depth 7</t>
+  </si>
+  <si>
+    <t>depth 8</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="9"/>
       <color theme="1"/>
@@ -77,13 +92,30 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="3">
@@ -130,16 +162,16 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -704,135 +736,234 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6AEAF64-B24F-4E2D-89CC-9E6FA66706DC}">
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr defaultRowHeight="12" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="18.83203125" style="6" customWidth="1"/>
-    <col min="2" max="16384" width="9.33203125" style="6"/>
+    <col min="1" max="1" width="18.83203125" style="1" customWidth="1"/>
+    <col min="2" max="16384" width="9.33203125" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" s="3">
-        <v>2</v>
-      </c>
-      <c r="C1" s="3">
-        <v>4</v>
-      </c>
-      <c r="D1" s="3">
+      <c r="A1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="5">
+        <v>2</v>
+      </c>
+      <c r="C1" s="5">
+        <v>4</v>
+      </c>
+      <c r="D1" s="5">
         <v>6</v>
       </c>
-      <c r="E1" s="3">
+      <c r="E1" s="5">
         <v>8</v>
       </c>
-      <c r="F1" s="3">
+      <c r="F1" s="5">
         <v>10</v>
       </c>
-      <c r="G1" s="3">
+      <c r="G1" s="5">
         <v>12</v>
       </c>
-      <c r="H1" s="3">
+      <c r="H1" s="5">
         <v>14</v>
       </c>
-      <c r="I1" s="3">
+      <c r="I1" s="5">
         <v>16</v>
       </c>
-      <c r="J1" s="3">
+      <c r="J1" s="5">
         <v>18</v>
       </c>
-      <c r="K1" s="5"/>
+      <c r="K1" s="4"/>
     </row>
     <row r="2" spans="1:11" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="4">
-        <v>1</v>
-      </c>
-      <c r="C2" s="4">
-        <v>2</v>
-      </c>
-      <c r="D2" s="4">
-        <v>2</v>
-      </c>
-      <c r="E2" s="4">
+      <c r="A2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="3">
+        <v>1</v>
+      </c>
+      <c r="C2" s="3">
+        <v>2</v>
+      </c>
+      <c r="D2" s="3">
+        <v>2</v>
+      </c>
+      <c r="E2" s="3">
         <v>3</v>
       </c>
-      <c r="F2" s="4">
+      <c r="F2" s="3">
         <v>3</v>
       </c>
-      <c r="G2" s="4">
-        <v>4</v>
-      </c>
-      <c r="H2" s="4">
-        <v>4</v>
-      </c>
-      <c r="I2" s="4">
+      <c r="G2" s="3">
+        <v>4</v>
+      </c>
+      <c r="H2" s="3">
+        <v>4</v>
+      </c>
+      <c r="I2" s="3">
         <v>5</v>
       </c>
-      <c r="J2" s="4">
+      <c r="J2" s="3">
         <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="4">
-        <v>1</v>
-      </c>
-      <c r="C3" s="4">
-        <v>2</v>
-      </c>
-      <c r="D3" s="4">
-        <v>4</v>
-      </c>
-      <c r="E3" s="4">
+      <c r="B3" s="3">
+        <v>1</v>
+      </c>
+      <c r="C3" s="3">
+        <v>2</v>
+      </c>
+      <c r="D3" s="3">
+        <v>4</v>
+      </c>
+      <c r="E3" s="3">
         <v>12</v>
       </c>
-      <c r="F3" s="4">
+      <c r="F3" s="3">
         <v>18</v>
       </c>
-      <c r="G3" s="4">
+      <c r="G3" s="3">
         <v>41</v>
       </c>
-      <c r="H3" s="4">
+      <c r="H3" s="3">
         <v>69</v>
       </c>
-      <c r="I3" s="4">
+      <c r="I3" s="3">
         <v>149</v>
       </c>
-      <c r="J3" s="4"/>
+      <c r="J3" s="3"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A4" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="4">
-        <v>1</v>
-      </c>
-      <c r="C4" s="4">
-        <v>1</v>
-      </c>
-      <c r="D4" s="4">
+      <c r="A4" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="3">
+        <v>1</v>
+      </c>
+      <c r="C4" s="3">
+        <v>1</v>
+      </c>
+      <c r="D4" s="3">
         <v>3</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="3">
         <v>13</v>
       </c>
-      <c r="F4" s="4">
+      <c r="F4" s="3">
         <v>171</v>
       </c>
-      <c r="G4" s="4">
+      <c r="G4" s="3">
         <v>1502</v>
       </c>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4"/>
+      <c r="H4" s="3">
+        <v>11108</v>
+      </c>
+      <c r="I4" s="3"/>
+      <c r="J4" s="6"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3">
+        <v>2</v>
+      </c>
+      <c r="E5" s="3">
+        <v>9</v>
+      </c>
+      <c r="F5" s="3">
+        <v>258</v>
+      </c>
+      <c r="G5" s="3">
+        <v>11753</v>
+      </c>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A6" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3">
+        <v>1</v>
+      </c>
+      <c r="E6" s="3">
+        <v>2</v>
+      </c>
+      <c r="F6" s="3">
+        <v>51</v>
+      </c>
+      <c r="G6" s="3">
+        <v>2164</v>
+      </c>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A7" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3">
+        <v>1</v>
+      </c>
+      <c r="F7" s="3">
+        <v>6</v>
+      </c>
+      <c r="G7" s="3">
+        <v>132</v>
+      </c>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="3"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A8" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3">
+        <v>1</v>
+      </c>
+      <c r="G8" s="3">
+        <v>5</v>
+      </c>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A9" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="3"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Multithread PrefixGenerator and start PrefixGeneratorV4.
</commit_message>
<xml_diff>
--- a/PrefixesV2.xlsx
+++ b/PrefixesV2.xlsx
@@ -8,14 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matty\source\repos\SortNetSAT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89035755-733E-4581-A32C-AACEB660DD18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EDB3278-F84B-4951-A25C-12B6C1FA7E58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0104B856-7785-45C9-88AA-D6349C4CC1CA}"/>
   </bookViews>
   <sheets>
     <sheet name="Combined" sheetId="9" r:id="rId1"/>
     <sheet name="Timings" sheetId="11" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="12" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="15">
   <si>
     <t>n</t>
   </si>
@@ -77,18 +76,6 @@
   </si>
   <si>
     <t>Descending Outputs</t>
-  </si>
-  <si>
-    <t>&lt;precheckRHS</t>
-  </si>
-  <si>
-    <t>&gt;precheckRHS</t>
-  </si>
-  <si>
-    <t>&lt;precheckLHS</t>
-  </si>
-  <si>
-    <t>&gt;precheckLHS</t>
   </si>
   <si>
     <t>Precheck:   236433764205</t>
@@ -171,7 +158,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -188,14 +175,8 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -767,18 +748,18 @@
       <c r="J9" s="2"/>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="I10" s="1" t="s">
-        <v>16</v>
+      <c r="I10" s="6" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="I11" s="1" t="s">
-        <v>17</v>
+      <c r="I11" s="6" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="I12" s="1" t="s">
-        <v>18</v>
+      <c r="I12" s="6" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -792,23 +773,23 @@
   <dimension ref="A1:K17"/>
   <sheetFormatPr defaultRowHeight="12" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="18.83203125" style="7" customWidth="1"/>
-    <col min="2" max="16384" width="9.33203125" style="7"/>
+    <col min="1" max="1" width="18.83203125" style="1" customWidth="1"/>
+    <col min="2" max="16384" width="9.33203125" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
-      <c r="I1" s="9"/>
-      <c r="J1" s="9"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="7"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
@@ -841,7 +822,7 @@
       <c r="J2" s="4">
         <v>18</v>
       </c>
-      <c r="K2" s="6"/>
+      <c r="K2" s="3"/>
     </row>
     <row r="3" spans="1:11" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
@@ -919,21 +900,21 @@
       </c>
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
-      <c r="J5" s="8"/>
+      <c r="J5" s="2"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A7" s="9" t="s">
+      <c r="A7" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="9"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
+      <c r="B7" s="7"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="7"/>
+      <c r="G7" s="7"/>
+      <c r="H7" s="7"/>
+      <c r="I7" s="7"/>
+      <c r="J7" s="7"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
@@ -1043,21 +1024,21 @@
       </c>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
-      <c r="J11" s="8"/>
+      <c r="J11" s="2"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A13" s="9" t="s">
+      <c r="A13" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="9"/>
-      <c r="C13" s="9"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="9"/>
-      <c r="G13" s="9"/>
-      <c r="H13" s="9"/>
-      <c r="I13" s="9"/>
-      <c r="J13" s="9"/>
+      <c r="B13" s="7"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="7"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="7"/>
+      <c r="H13" s="7"/>
+      <c r="I13" s="7"/>
+      <c r="J13" s="7"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
@@ -1173,7 +1154,7 @@
       <c r="I17" s="2">
         <v>13007.462578999999</v>
       </c>
-      <c r="J17" s="8"/>
+      <c r="J17" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1183,45 +1164,4 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7B66B4B-D3B5-43FD-A975-CFAA26AA6836}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="12" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="4" width="13.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2">
-        <v>3.8492057000000002</v>
-      </c>
-      <c r="B2">
-        <v>7.7777791000000001</v>
-      </c>
-      <c r="C2">
-        <v>10.6830879</v>
-      </c>
-      <c r="D2">
-        <v>5.1965969999999997</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Don't use two-phase pruning. Implement BulkChecker.
</commit_message>
<xml_diff>
--- a/PrefixesV2.xlsx
+++ b/PrefixesV2.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matty\source\repos\SortNetSAT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EDB3278-F84B-4951-A25C-12B6C1FA7E58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4940D48-60E0-4DE9-BB6D-E7E4B58358FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0104B856-7785-45C9-88AA-D6349C4CC1CA}"/>
   </bookViews>
   <sheets>
-    <sheet name="Combined" sheetId="9" r:id="rId1"/>
-    <sheet name="Timings" sheetId="11" r:id="rId2"/>
+    <sheet name="CombinedSym" sheetId="9" r:id="rId1"/>
+    <sheet name="CombinedUnsym" sheetId="12" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="9">
   <si>
     <t>n</t>
   </si>
@@ -68,30 +68,12 @@
   <si>
     <t>depth 8</t>
   </si>
-  <si>
-    <t>Random Order</t>
-  </si>
-  <si>
-    <t>Ascending Outputs</t>
-  </si>
-  <si>
-    <t>Descending Outputs</t>
-  </si>
-  <si>
-    <t>Precheck:   236433764205</t>
-  </si>
-  <si>
-    <t>Restricted: 84431931</t>
-  </si>
-  <si>
-    <t>Full:       36869242</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="9"/>
       <color theme="1"/>
@@ -107,6 +89,17 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -158,7 +151,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -178,8 +171,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -647,7 +649,9 @@
       <c r="I4" s="2">
         <v>92963</v>
       </c>
-      <c r="J4" s="5"/>
+      <c r="J4" s="5">
+        <v>749749</v>
+      </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
@@ -748,19 +752,13 @@
       <c r="J9" s="2"/>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="I10" s="6" t="s">
-        <v>12</v>
-      </c>
+      <c r="I10" s="6"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="I11" s="6" t="s">
-        <v>13</v>
-      </c>
+      <c r="I11" s="6"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="I12" s="6" t="s">
-        <v>14</v>
-      </c>
+      <c r="I12" s="6"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -769,399 +767,330 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20E317F0-04C5-466D-A9D7-E11764D05689}">
-  <dimension ref="A1:K17"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFEC3168-15A0-41D9-B6E3-174A23AA57D1}">
+  <dimension ref="A1:P12"/>
   <sheetFormatPr defaultRowHeight="12" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="18.83203125" style="1" customWidth="1"/>
-    <col min="2" max="16384" width="9.33203125" style="1"/>
+    <col min="1" max="1" width="18.83203125" style="9" customWidth="1"/>
+    <col min="2" max="16384" width="9.33203125" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A1" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="8">
+        <v>2</v>
+      </c>
+      <c r="C1" s="8">
+        <v>3</v>
+      </c>
+      <c r="D1" s="8">
+        <v>4</v>
+      </c>
+      <c r="E1" s="8">
+        <v>5</v>
+      </c>
+      <c r="F1" s="8">
+        <v>6</v>
+      </c>
+      <c r="G1" s="8">
+        <v>7</v>
+      </c>
+      <c r="H1" s="8">
+        <v>8</v>
+      </c>
+      <c r="I1" s="8">
         <v>9</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
-      <c r="I1" s="7"/>
-      <c r="J1" s="7"/>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="4">
-        <v>2</v>
-      </c>
-      <c r="C2" s="4">
+      <c r="J1" s="8">
+        <v>10</v>
+      </c>
+      <c r="K1" s="8">
+        <v>11</v>
+      </c>
+      <c r="L1" s="8">
+        <v>12</v>
+      </c>
+      <c r="M1" s="8">
+        <v>13</v>
+      </c>
+      <c r="N1" s="8">
+        <v>14</v>
+      </c>
+      <c r="O1" s="8">
+        <v>15</v>
+      </c>
+      <c r="P1" s="8">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="7">
+        <v>1</v>
+      </c>
+      <c r="C2" s="7">
+        <v>1</v>
+      </c>
+      <c r="D2" s="7">
+        <v>1</v>
+      </c>
+      <c r="E2" s="7">
+        <v>1</v>
+      </c>
+      <c r="F2" s="7">
+        <v>1</v>
+      </c>
+      <c r="G2" s="7">
+        <v>1</v>
+      </c>
+      <c r="H2" s="7">
+        <v>1</v>
+      </c>
+      <c r="I2" s="7">
+        <v>1</v>
+      </c>
+      <c r="J2" s="7">
+        <v>1</v>
+      </c>
+      <c r="K2" s="7">
+        <v>1</v>
+      </c>
+      <c r="L2" s="7">
+        <v>1</v>
+      </c>
+      <c r="M2" s="7">
+        <v>1</v>
+      </c>
+      <c r="N2" s="7">
+        <v>1</v>
+      </c>
+      <c r="O2" s="7">
+        <v>1</v>
+      </c>
+      <c r="P2" s="7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A3" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="7"/>
+      <c r="C3" s="7">
+        <v>2</v>
+      </c>
+      <c r="D3" s="7">
+        <v>2</v>
+      </c>
+      <c r="E3" s="7">
+        <v>6</v>
+      </c>
+      <c r="F3" s="7">
+        <v>6</v>
+      </c>
+      <c r="G3" s="7">
+        <v>14</v>
+      </c>
+      <c r="H3" s="7">
+        <v>15</v>
+      </c>
+      <c r="I3" s="7">
+        <v>37</v>
+      </c>
+      <c r="J3" s="7">
+        <v>27</v>
+      </c>
+      <c r="K3" s="7">
+        <v>88</v>
+      </c>
+      <c r="L3" s="7">
+        <v>70</v>
+      </c>
+      <c r="M3" s="7"/>
+      <c r="N3" s="7"/>
+      <c r="O3" s="7"/>
+      <c r="P3" s="7"/>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A4" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="7"/>
+      <c r="C4" s="7">
+        <v>1</v>
+      </c>
+      <c r="D4" s="7">
+        <v>1</v>
+      </c>
+      <c r="E4" s="7">
+        <v>7</v>
+      </c>
+      <c r="F4" s="7">
+        <v>5</v>
+      </c>
+      <c r="G4" s="7">
+        <v>99</v>
+      </c>
+      <c r="H4" s="7">
+        <v>68</v>
+      </c>
+      <c r="I4" s="7">
+        <v>3090</v>
+      </c>
+      <c r="J4" s="7">
+        <v>6176</v>
+      </c>
+      <c r="K4" s="7">
+        <v>111307</v>
+      </c>
+      <c r="L4" s="7"/>
+      <c r="M4" s="7"/>
+      <c r="N4" s="7"/>
+      <c r="O4" s="7"/>
+      <c r="P4" s="7"/>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A5" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="4">
+      <c r="B5" s="7"/>
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7">
+        <v>2</v>
+      </c>
+      <c r="F5" s="7">
+        <v>2</v>
+      </c>
+      <c r="G5" s="7">
+        <v>30</v>
+      </c>
+      <c r="H5" s="7">
+        <v>28</v>
+      </c>
+      <c r="I5" s="7">
+        <v>6460</v>
+      </c>
+      <c r="J5" s="7"/>
+      <c r="K5" s="7"/>
+      <c r="L5" s="7"/>
+      <c r="M5" s="7"/>
+      <c r="N5" s="7"/>
+      <c r="O5" s="7"/>
+      <c r="P5" s="7"/>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A6" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="7"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7">
+        <v>1</v>
+      </c>
+      <c r="F6" s="7">
+        <v>1</v>
+      </c>
+      <c r="G6" s="7">
+        <v>3</v>
+      </c>
+      <c r="H6" s="7">
+        <v>4</v>
+      </c>
+      <c r="I6" s="7">
+        <v>396</v>
+      </c>
+      <c r="J6" s="7"/>
+      <c r="K6" s="7"/>
+      <c r="L6" s="7"/>
+      <c r="M6" s="7"/>
+      <c r="N6" s="7"/>
+      <c r="O6" s="7"/>
+      <c r="P6" s="7"/>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A7" s="7" t="s">
         <v>6</v>
-      </c>
-      <c r="E2" s="4">
-        <v>8</v>
-      </c>
-      <c r="F2" s="4">
-        <v>10</v>
-      </c>
-      <c r="G2" s="4">
-        <v>12</v>
-      </c>
-      <c r="H2" s="4">
-        <v>14</v>
-      </c>
-      <c r="I2" s="4">
-        <v>16</v>
-      </c>
-      <c r="J2" s="4">
-        <v>18</v>
-      </c>
-      <c r="K2" s="3"/>
-    </row>
-    <row r="3" spans="1:11" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="2">
-        <v>7.79667E-5</v>
-      </c>
-      <c r="C3" s="2">
-        <v>7.1233299999999994E-5</v>
-      </c>
-      <c r="D3" s="2">
-        <v>2.198333E-4</v>
-      </c>
-      <c r="E3" s="2">
-        <v>4.4030000000000002E-4</v>
-      </c>
-      <c r="F3" s="2">
-        <v>2.7013332999999999E-3</v>
-      </c>
-      <c r="G3" s="2">
-        <v>5.87349333E-2</v>
-      </c>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A4" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="2">
-        <v>4.9866700000000001E-5</v>
-      </c>
-      <c r="C4" s="2">
-        <v>7.7766699999999995E-5</v>
-      </c>
-      <c r="D4" s="2">
-        <v>1.6990000000000001E-4</v>
-      </c>
-      <c r="E4" s="2">
-        <v>1.5863333E-3</v>
-      </c>
-      <c r="F4" s="2">
-        <v>1.5214066700000001E-2</v>
-      </c>
-      <c r="G4" s="2">
-        <v>0.57605126669999995</v>
-      </c>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A5" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="2">
-        <v>5.2299999999999997E-5</v>
-      </c>
-      <c r="C5" s="2">
-        <v>6.1366700000000003E-5</v>
-      </c>
-      <c r="D5" s="2">
-        <v>2.0976670000000001E-4</v>
-      </c>
-      <c r="E5" s="2">
-        <v>4.6279666999999997E-3</v>
-      </c>
-      <c r="F5" s="2">
-        <v>8.9779033300000005E-2</v>
-      </c>
-      <c r="G5" s="2">
-        <v>7.2977490666999998</v>
-      </c>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A7" s="7" t="s">
-        <v>10</v>
       </c>
       <c r="B7" s="7"/>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
       <c r="E7" s="7"/>
       <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
-      <c r="H7" s="7"/>
-      <c r="I7" s="7"/>
+      <c r="G7" s="7">
+        <v>1</v>
+      </c>
+      <c r="H7" s="7">
+        <v>1</v>
+      </c>
+      <c r="I7" s="7">
+        <v>12</v>
+      </c>
       <c r="J7" s="7"/>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A8" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="B8" s="4">
-        <v>2</v>
-      </c>
-      <c r="C8" s="4">
-        <v>4</v>
-      </c>
-      <c r="D8" s="4">
-        <v>6</v>
-      </c>
-      <c r="E8" s="4">
+      <c r="K7" s="7"/>
+      <c r="L7" s="7"/>
+      <c r="M7" s="7"/>
+      <c r="N7" s="7"/>
+      <c r="O7" s="7"/>
+      <c r="P7" s="7"/>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A8" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="7"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="7"/>
+      <c r="H8" s="7"/>
+      <c r="I8" s="7">
+        <v>1</v>
+      </c>
+      <c r="J8" s="7"/>
+      <c r="K8" s="7"/>
+      <c r="L8" s="7"/>
+      <c r="M8" s="7"/>
+      <c r="N8" s="7"/>
+      <c r="O8" s="7"/>
+      <c r="P8" s="7"/>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A9" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="F8" s="4">
-        <v>10</v>
-      </c>
-      <c r="G8" s="4">
-        <v>12</v>
-      </c>
-      <c r="H8" s="4">
-        <v>14</v>
-      </c>
-      <c r="I8" s="4">
-        <v>16</v>
-      </c>
-      <c r="J8" s="4">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A9" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B9" s="2">
-        <v>1.571333E-4</v>
-      </c>
-      <c r="C9" s="2">
-        <v>6.9666700000000002E-5</v>
-      </c>
-      <c r="D9" s="2">
-        <v>9.6766699999999996E-5</v>
-      </c>
-      <c r="E9" s="2">
-        <v>4.1696669999999997E-4</v>
-      </c>
-      <c r="F9" s="2">
-        <v>4.7904000000000002E-3</v>
-      </c>
-      <c r="G9" s="2">
-        <v>9.7388333300000005E-2</v>
-      </c>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2"/>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A10" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B10" s="2">
-        <v>6.1799999999999998E-5</v>
-      </c>
-      <c r="C10" s="2">
-        <v>7.6299999999999998E-5</v>
-      </c>
-      <c r="D10" s="2">
-        <v>1.804667E-4</v>
-      </c>
-      <c r="E10" s="2">
-        <v>2.4757999999999998E-3</v>
-      </c>
-      <c r="F10" s="2">
-        <v>3.2995233300000003E-2</v>
-      </c>
-      <c r="G10" s="2">
-        <v>1.1942296333</v>
-      </c>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
-      <c r="J10" s="2"/>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A11" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" s="2">
-        <v>5.75333E-5</v>
-      </c>
-      <c r="C11" s="2">
-        <v>5.9933299999999998E-5</v>
-      </c>
-      <c r="D11" s="2">
-        <v>1.8196670000000001E-4</v>
-      </c>
-      <c r="E11" s="2">
-        <v>5.2655667E-3</v>
-      </c>
-      <c r="F11" s="2">
-        <v>0.1247981667</v>
-      </c>
-      <c r="G11" s="2">
-        <v>12.198535166699999</v>
-      </c>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
-      <c r="J11" s="2"/>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A13" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B13" s="7"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="7"/>
-      <c r="H13" s="7"/>
-      <c r="I13" s="7"/>
-      <c r="J13" s="7"/>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A14" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="B14" s="4">
-        <v>2</v>
-      </c>
-      <c r="C14" s="4">
-        <v>4</v>
-      </c>
-      <c r="D14" s="4">
-        <v>6</v>
-      </c>
-      <c r="E14" s="4">
-        <v>8</v>
-      </c>
-      <c r="F14" s="4">
-        <v>10</v>
-      </c>
-      <c r="G14" s="4">
-        <v>12</v>
-      </c>
-      <c r="H14" s="4">
-        <v>14</v>
-      </c>
-      <c r="I14" s="4">
-        <v>16</v>
-      </c>
-      <c r="J14" s="4">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A15" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B15" s="2">
-        <v>8.1066699999999994E-5</v>
-      </c>
-      <c r="C15" s="2">
-        <v>7.7299999999999995E-5</v>
-      </c>
-      <c r="D15" s="2">
-        <v>1.3899999999999999E-4</v>
-      </c>
-      <c r="E15" s="2">
-        <v>4.3483330000000002E-4</v>
-      </c>
-      <c r="F15" s="2">
-        <v>3.6426666999999999E-3</v>
-      </c>
-      <c r="G15" s="2">
-        <v>8.0933466699999998E-2</v>
-      </c>
-      <c r="H15" s="2"/>
-      <c r="I15" s="2">
-        <v>40.077207799999996</v>
-      </c>
-      <c r="J15" s="2"/>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A16" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B16" s="2">
-        <v>6.6666699999999996E-5</v>
-      </c>
-      <c r="C16" s="2">
-        <v>9.2833300000000004E-5</v>
-      </c>
-      <c r="D16" s="2">
-        <v>1.9026669999999999E-4</v>
-      </c>
-      <c r="E16" s="2">
-        <v>1.6236E-3</v>
-      </c>
-      <c r="F16" s="2">
-        <v>1.14928667E-2</v>
-      </c>
-      <c r="G16" s="2">
-        <v>0.15692326670000001</v>
-      </c>
-      <c r="H16" s="2"/>
-      <c r="I16" s="2">
-        <v>33.068185200000002</v>
-      </c>
-      <c r="J16" s="2"/>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A17" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B17" s="2">
-        <v>6.3266699999999995E-5</v>
-      </c>
-      <c r="C17" s="2">
-        <v>8.1033300000000002E-5</v>
-      </c>
-      <c r="D17" s="2">
-        <v>2.1163329999999999E-4</v>
-      </c>
-      <c r="E17" s="2">
-        <v>4.2445666999999998E-3</v>
-      </c>
-      <c r="F17" s="2">
-        <v>5.1684533300000002E-2</v>
-      </c>
-      <c r="G17" s="2">
-        <v>1.8055611332999999</v>
-      </c>
-      <c r="H17" s="2"/>
-      <c r="I17" s="2">
-        <v>13007.462578999999</v>
-      </c>
-      <c r="J17" s="2"/>
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="7"/>
+      <c r="I9" s="7"/>
+      <c r="J9" s="7"/>
+      <c r="K9" s="7"/>
+      <c r="L9" s="7"/>
+      <c r="M9" s="7"/>
+      <c r="N9" s="7"/>
+      <c r="O9" s="7"/>
+      <c r="P9" s="7"/>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="I10" s="10"/>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="I11" s="10"/>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="I12" s="10"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A7:J7"/>
-    <mergeCell ref="A13:J13"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>